<commit_message>
feat: add F1-score calculation logic and export performance comparison plots for wound analysis categories
</commit_message>
<xml_diff>
--- a/exports/Lohmann_Rauscher_Vergleich_Experten_KI.xlsx
+++ b/exports/Lohmann_Rauscher_Vergleich_Experten_KI.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10802"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mertakdemir/Developer/uni/Modell/exports/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{202622D0-07AA-D54B-A320-5257A30ADB90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B113DF54-9AAB-7946-BA2D-3EA8A336B495}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="28200" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,7 +18,20 @@
     <sheet name="KI-Antworten" sheetId="4" r:id="rId3"/>
     <sheet name="Alle im Vergleich" sheetId="1" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -5845,21 +5858,25 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FF0F172A"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="9">
@@ -32882,15 +32899,6 @@
     </row>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="A6:A8"/>
-    <mergeCell ref="A3:A5"/>
-    <mergeCell ref="A42:A44"/>
-    <mergeCell ref="A18:A20"/>
-    <mergeCell ref="A27:A29"/>
-    <mergeCell ref="A9:A11"/>
-    <mergeCell ref="A36:A38"/>
-    <mergeCell ref="A30:A32"/>
-    <mergeCell ref="A39:A41"/>
     <mergeCell ref="A45:A47"/>
     <mergeCell ref="A21:A23"/>
     <mergeCell ref="A12:A14"/>
@@ -32901,6 +32909,15 @@
     <mergeCell ref="A48:A50"/>
     <mergeCell ref="A51:A53"/>
     <mergeCell ref="A54:A56"/>
+    <mergeCell ref="A6:A8"/>
+    <mergeCell ref="A3:A5"/>
+    <mergeCell ref="A42:A44"/>
+    <mergeCell ref="A18:A20"/>
+    <mergeCell ref="A27:A29"/>
+    <mergeCell ref="A9:A11"/>
+    <mergeCell ref="A36:A38"/>
+    <mergeCell ref="A30:A32"/>
+    <mergeCell ref="A39:A41"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing r:id="rId1"/>
@@ -50883,6 +50900,9 @@
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="A63:A67"/>
+    <mergeCell ref="A28:A32"/>
+    <mergeCell ref="A13:A17"/>
     <mergeCell ref="A3:A7"/>
     <mergeCell ref="A93:A97"/>
     <mergeCell ref="A73:A77"/>
@@ -50899,9 +50919,6 @@
     <mergeCell ref="A8:A12"/>
     <mergeCell ref="A33:A37"/>
     <mergeCell ref="A23:A27"/>
-    <mergeCell ref="A63:A67"/>
-    <mergeCell ref="A28:A32"/>
-    <mergeCell ref="A13:A17"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
feat: export extensive medical normalization mapping documentation and generate additional heatmap visualization assets
</commit_message>
<xml_diff>
--- a/exports/Lohmann_Rauscher_Vergleich_Experten_KI.xlsx
+++ b/exports/Lohmann_Rauscher_Vergleich_Experten_KI.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10802"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mertakdemir/Developer/uni/Modell/exports/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B113DF54-9AAB-7946-BA2D-3EA8A336B495}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5C57672-2B18-3C4A-87A4-A951FB385958}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="28200" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,6 +18,9 @@
     <sheet name="KI-Antworten" sheetId="4" r:id="rId3"/>
     <sheet name="Alle im Vergleich" sheetId="1" r:id="rId4"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm.Print_Titles" localSheetId="3">'Alle im Vergleich'!$A:$B,'Alle im Vergleich'!$1:$1</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -5845,7 +5848,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -14306,14 +14309,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:BJ21"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
     <col min="3" max="62" width="36" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:62" ht="25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:62" ht="25" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -14501,7 +14504,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="2" spans="1:62" ht="140" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:62" ht="140" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>62</v>
       </c>
@@ -14569,7 +14572,7 @@
       <c r="BI2" s="4"/>
       <c r="BJ2" s="4"/>
     </row>
-    <row r="3" spans="1:62" ht="45" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:62" ht="45">
       <c r="A3" s="15" t="s">
         <v>64</v>
       </c>
@@ -14757,7 +14760,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="4" spans="1:62" ht="16" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:62" ht="16">
       <c r="A4" s="15" t="s">
         <v>324</v>
       </c>
@@ -14945,7 +14948,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="5" spans="1:62" ht="30" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:62" ht="30">
       <c r="A5" s="15" t="s">
         <v>560</v>
       </c>
@@ -15133,7 +15136,7 @@
         <v>570</v>
       </c>
     </row>
-    <row r="6" spans="1:62" ht="45" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:62" ht="45">
       <c r="A6" s="15" t="s">
         <v>611</v>
       </c>
@@ -15321,7 +15324,7 @@
         <v>648</v>
       </c>
     </row>
-    <row r="7" spans="1:62" ht="30" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:62" ht="30">
       <c r="A7" s="15" t="s">
         <v>877</v>
       </c>
@@ -15509,7 +15512,7 @@
         <v>885</v>
       </c>
     </row>
-    <row r="8" spans="1:62" ht="45" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:62" ht="45">
       <c r="A8" s="15" t="s">
         <v>924</v>
       </c>
@@ -15697,7 +15700,7 @@
         <v>926</v>
       </c>
     </row>
-    <row r="9" spans="1:62" ht="30" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:62" ht="30">
       <c r="A9" s="15" t="s">
         <v>971</v>
       </c>
@@ -15885,7 +15888,7 @@
         <v>997</v>
       </c>
     </row>
-    <row r="10" spans="1:62" ht="60" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:62" ht="60">
       <c r="A10" s="15" t="s">
         <v>1033</v>
       </c>
@@ -16073,7 +16076,7 @@
         <v>1050</v>
       </c>
     </row>
-    <row r="11" spans="1:62" ht="16" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:62" ht="16">
       <c r="A11" s="15" t="s">
         <v>1263</v>
       </c>
@@ -16261,7 +16264,7 @@
         <v>1264</v>
       </c>
     </row>
-    <row r="12" spans="1:62" ht="16" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:62" ht="16">
       <c r="A12" s="15" t="s">
         <v>1268</v>
       </c>
@@ -16449,7 +16452,7 @@
         <v>1278</v>
       </c>
     </row>
-    <row r="13" spans="1:62" ht="16" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:62" ht="16">
       <c r="A13" s="15" t="s">
         <v>1321</v>
       </c>
@@ -16637,7 +16640,7 @@
         <v>1265</v>
       </c>
     </row>
-    <row r="14" spans="1:62" ht="16" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:62" ht="16">
       <c r="A14" s="15" t="s">
         <v>1322</v>
       </c>
@@ -16825,7 +16828,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="15" spans="1:62" ht="30" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:62" ht="30">
       <c r="A15" s="15" t="s">
         <v>1325</v>
       </c>
@@ -17013,7 +17016,7 @@
         <v>1326</v>
       </c>
     </row>
-    <row r="16" spans="1:62" ht="30" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:62" ht="30">
       <c r="A16" s="15" t="s">
         <v>1455</v>
       </c>
@@ -17201,7 +17204,7 @@
         <v>1338</v>
       </c>
     </row>
-    <row r="17" spans="1:62" ht="16" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:62" ht="16">
       <c r="A17" s="15" t="s">
         <v>1558</v>
       </c>
@@ -17389,7 +17392,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="18" spans="1:62" ht="16" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:62" ht="16">
       <c r="A18" s="15" t="s">
         <v>1616</v>
       </c>
@@ -17577,7 +17580,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="19" spans="1:62" ht="16" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:62" ht="16">
       <c r="A19" s="15" t="s">
         <v>1653</v>
       </c>
@@ -17765,7 +17768,7 @@
         <v>1265</v>
       </c>
     </row>
-    <row r="20" spans="1:62" ht="30" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:62" ht="30">
       <c r="A20" s="15" t="s">
         <v>1655</v>
       </c>
@@ -17953,7 +17956,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="21" spans="1:62" ht="75" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:62" ht="75">
       <c r="A21" s="15" t="s">
         <v>1678</v>
       </c>
@@ -18143,6 +18146,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
@@ -18150,14 +18154,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:BJ21"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
     <col min="3" max="62" width="36" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:62" ht="25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:62" ht="25" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -18345,7 +18349,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="2" spans="1:62" ht="140" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:62" ht="140" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>62</v>
       </c>
@@ -18413,7 +18417,7 @@
       <c r="BI2" s="4"/>
       <c r="BJ2" s="4"/>
     </row>
-    <row r="3" spans="1:62" ht="75" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:62" ht="75">
       <c r="A3" s="18" t="s">
         <v>64</v>
       </c>
@@ -18601,7 +18605,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="4" spans="1:62" ht="45" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:62" ht="45">
       <c r="A4" s="18" t="s">
         <v>324</v>
       </c>
@@ -18789,7 +18793,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="5" spans="1:62" ht="30" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:62" ht="30">
       <c r="A5" s="18" t="s">
         <v>560</v>
       </c>
@@ -18977,7 +18981,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="6" spans="1:62" ht="75" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:62" ht="75">
       <c r="A6" s="18" t="s">
         <v>611</v>
       </c>
@@ -19165,7 +19169,7 @@
         <v>698</v>
       </c>
     </row>
-    <row r="7" spans="1:62" ht="30" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:62" ht="30">
       <c r="A7" s="18" t="s">
         <v>877</v>
       </c>
@@ -19353,7 +19357,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="8" spans="1:62" ht="45" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:62" ht="45">
       <c r="A8" s="18" t="s">
         <v>924</v>
       </c>
@@ -19541,7 +19545,7 @@
         <v>925</v>
       </c>
     </row>
-    <row r="9" spans="1:62" ht="45" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:62" ht="45">
       <c r="A9" s="18" t="s">
         <v>971</v>
       </c>
@@ -19729,7 +19733,7 @@
         <v>1027</v>
       </c>
     </row>
-    <row r="10" spans="1:62" ht="150" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:62" ht="150">
       <c r="A10" s="18" t="s">
         <v>1033</v>
       </c>
@@ -19917,7 +19921,7 @@
         <v>1105</v>
       </c>
     </row>
-    <row r="11" spans="1:62" ht="16" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:62" ht="16">
       <c r="A11" s="18" t="s">
         <v>1263</v>
       </c>
@@ -20105,7 +20109,7 @@
         <v>1264</v>
       </c>
     </row>
-    <row r="12" spans="1:62" ht="30" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:62" ht="30">
       <c r="A12" s="18" t="s">
         <v>1268</v>
       </c>
@@ -20293,7 +20297,7 @@
         <v>1293</v>
       </c>
     </row>
-    <row r="13" spans="1:62" ht="16" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:62" ht="16">
       <c r="A13" s="18" t="s">
         <v>1321</v>
       </c>
@@ -20481,7 +20485,7 @@
         <v>1264</v>
       </c>
     </row>
-    <row r="14" spans="1:62" ht="16" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:62" ht="16">
       <c r="A14" s="18" t="s">
         <v>1322</v>
       </c>
@@ -20669,7 +20673,7 @@
         <v>1324</v>
       </c>
     </row>
-    <row r="15" spans="1:62" ht="30" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:62" ht="30">
       <c r="A15" s="18" t="s">
         <v>1325</v>
       </c>
@@ -20857,7 +20861,7 @@
         <v>1354</v>
       </c>
     </row>
-    <row r="16" spans="1:62" ht="30" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:62" ht="30">
       <c r="A16" s="18" t="s">
         <v>1455</v>
       </c>
@@ -21045,7 +21049,7 @@
         <v>1475</v>
       </c>
     </row>
-    <row r="17" spans="1:62" ht="16" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:62" ht="16">
       <c r="A17" s="18" t="s">
         <v>1558</v>
       </c>
@@ -21233,7 +21237,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="18" spans="1:62" ht="16" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:62" ht="16">
       <c r="A18" s="18" t="s">
         <v>1616</v>
       </c>
@@ -21421,7 +21425,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="19" spans="1:62" ht="16" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:62" ht="16">
       <c r="A19" s="18" t="s">
         <v>1653</v>
       </c>
@@ -21609,7 +21613,7 @@
         <v>1265</v>
       </c>
     </row>
-    <row r="20" spans="1:62" ht="45" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:62" ht="45">
       <c r="A20" s="18" t="s">
         <v>1655</v>
       </c>
@@ -21797,7 +21801,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="21" spans="1:62" ht="105" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:62" ht="105">
       <c r="A21" s="18" t="s">
         <v>1678</v>
       </c>
@@ -21987,6 +21991,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
@@ -21994,14 +21999,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:BJ59"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
     <col min="3" max="62" width="36" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:62" ht="25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:62" ht="25" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -22189,7 +22194,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="2" spans="1:62" ht="140" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:62" ht="140" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>62</v>
       </c>
@@ -22257,7 +22262,7 @@
       <c r="BI2" s="4"/>
       <c r="BJ2" s="4"/>
     </row>
-    <row r="3" spans="1:62" ht="45" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:62" ht="45">
       <c r="A3" s="24" t="s">
         <v>64</v>
       </c>
@@ -22445,7 +22450,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="4" spans="1:62" ht="45" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:62" ht="45">
       <c r="A4" s="22"/>
       <c r="B4" s="11" t="s">
         <v>224</v>
@@ -22631,7 +22636,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="5" spans="1:62" ht="30" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:62" ht="30">
       <c r="A5" s="23"/>
       <c r="B5" s="13" t="s">
         <v>280</v>
@@ -22817,7 +22822,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="6" spans="1:62" ht="30" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:62" ht="30">
       <c r="A6" s="24" t="s">
         <v>324</v>
       </c>
@@ -23005,7 +23010,7 @@
         <v>461</v>
       </c>
     </row>
-    <row r="7" spans="1:62" ht="30" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:62" ht="30">
       <c r="A7" s="22"/>
       <c r="B7" s="11" t="s">
         <v>224</v>
@@ -23191,7 +23196,7 @@
         <v>502</v>
       </c>
     </row>
-    <row r="8" spans="1:62" ht="60" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:62" ht="60">
       <c r="A8" s="23"/>
       <c r="B8" s="13" t="s">
         <v>280</v>
@@ -23377,7 +23382,7 @@
         <v>559</v>
       </c>
     </row>
-    <row r="9" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:62">
       <c r="A9" s="24" t="s">
         <v>560</v>
       </c>
@@ -23565,7 +23570,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="10" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:62">
       <c r="A10" s="22"/>
       <c r="B10" s="11" t="s">
         <v>224</v>
@@ -23751,7 +23756,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="11" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:62">
       <c r="A11" s="23"/>
       <c r="B11" s="13" t="s">
         <v>280</v>
@@ -23937,7 +23942,7 @@
         <v>610</v>
       </c>
     </row>
-    <row r="12" spans="1:62" ht="75" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:62" ht="75">
       <c r="A12" s="24" t="s">
         <v>611</v>
       </c>
@@ -24125,7 +24130,7 @@
         <v>758</v>
       </c>
     </row>
-    <row r="13" spans="1:62" ht="60" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:62" ht="60">
       <c r="A13" s="22"/>
       <c r="B13" s="11" t="s">
         <v>224</v>
@@ -24311,7 +24316,7 @@
         <v>816</v>
       </c>
     </row>
-    <row r="14" spans="1:62" ht="120" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:62" ht="120">
       <c r="A14" s="23"/>
       <c r="B14" s="13" t="s">
         <v>280</v>
@@ -24497,7 +24502,7 @@
         <v>876</v>
       </c>
     </row>
-    <row r="15" spans="1:62" ht="30" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:62" ht="30">
       <c r="A15" s="24" t="s">
         <v>877</v>
       </c>
@@ -24685,7 +24690,7 @@
         <v>903</v>
       </c>
     </row>
-    <row r="16" spans="1:62" ht="30" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:62" ht="30">
       <c r="A16" s="22"/>
       <c r="B16" s="11" t="s">
         <v>224</v>
@@ -24871,7 +24876,7 @@
         <v>904</v>
       </c>
     </row>
-    <row r="17" spans="1:62" ht="30" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:62" ht="30">
       <c r="A17" s="23"/>
       <c r="B17" s="13" t="s">
         <v>280</v>
@@ -25057,7 +25062,7 @@
         <v>904</v>
       </c>
     </row>
-    <row r="18" spans="1:62" ht="60" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:62" ht="60">
       <c r="A18" s="24" t="s">
         <v>924</v>
       </c>
@@ -25245,7 +25250,7 @@
         <v>957</v>
       </c>
     </row>
-    <row r="19" spans="1:62" ht="45" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:62" ht="45">
       <c r="A19" s="22"/>
       <c r="B19" s="11" t="s">
         <v>224</v>
@@ -25431,7 +25436,7 @@
         <v>954</v>
       </c>
     </row>
-    <row r="20" spans="1:62" ht="60" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:62" ht="60">
       <c r="A20" s="23"/>
       <c r="B20" s="13" t="s">
         <v>280</v>
@@ -25617,7 +25622,7 @@
         <v>954</v>
       </c>
     </row>
-    <row r="21" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:62">
       <c r="A21" s="24" t="s">
         <v>971</v>
       </c>
@@ -25805,7 +25810,7 @@
         <v>1030</v>
       </c>
     </row>
-    <row r="22" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:62">
       <c r="A22" s="22"/>
       <c r="B22" s="11" t="s">
         <v>224</v>
@@ -25991,7 +25996,7 @@
         <v>1030</v>
       </c>
     </row>
-    <row r="23" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:62">
       <c r="A23" s="23"/>
       <c r="B23" s="13" t="s">
         <v>280</v>
@@ -26177,7 +26182,7 @@
         <v>1030</v>
       </c>
     </row>
-    <row r="24" spans="1:62" ht="60" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:62" ht="60">
       <c r="A24" s="24" t="s">
         <v>1033</v>
       </c>
@@ -26365,7 +26370,7 @@
         <v>1153</v>
       </c>
     </row>
-    <row r="25" spans="1:62" ht="60" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:62" ht="60">
       <c r="A25" s="22"/>
       <c r="B25" s="11" t="s">
         <v>224</v>
@@ -26551,7 +26556,7 @@
         <v>1210</v>
       </c>
     </row>
-    <row r="26" spans="1:62" ht="75" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:62" ht="75">
       <c r="A26" s="23"/>
       <c r="B26" s="13" t="s">
         <v>280</v>
@@ -26737,7 +26742,7 @@
         <v>1262</v>
       </c>
     </row>
-    <row r="27" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:62">
       <c r="A27" s="24" t="s">
         <v>1263</v>
       </c>
@@ -26925,7 +26930,7 @@
         <v>1266</v>
       </c>
     </row>
-    <row r="28" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:62">
       <c r="A28" s="22"/>
       <c r="B28" s="11" t="s">
         <v>224</v>
@@ -27111,7 +27116,7 @@
         <v>1266</v>
       </c>
     </row>
-    <row r="29" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:62">
       <c r="A29" s="23"/>
       <c r="B29" s="13" t="s">
         <v>280</v>
@@ -27297,7 +27302,7 @@
         <v>1266</v>
       </c>
     </row>
-    <row r="30" spans="1:62" ht="30" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:62" ht="30">
       <c r="A30" s="24" t="s">
         <v>1268</v>
       </c>
@@ -27485,7 +27490,7 @@
         <v>1301</v>
       </c>
     </row>
-    <row r="31" spans="1:62" ht="30" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:62" ht="30">
       <c r="A31" s="22"/>
       <c r="B31" s="11" t="s">
         <v>224</v>
@@ -27671,7 +27676,7 @@
         <v>1302</v>
       </c>
     </row>
-    <row r="32" spans="1:62" ht="45" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:62" ht="45">
       <c r="A32" s="23"/>
       <c r="B32" s="13" t="s">
         <v>280</v>
@@ -27857,7 +27862,7 @@
         <v>1301</v>
       </c>
     </row>
-    <row r="33" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:62">
       <c r="A33" s="24" t="s">
         <v>1321</v>
       </c>
@@ -28045,7 +28050,7 @@
         <v>1267</v>
       </c>
     </row>
-    <row r="34" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:62">
       <c r="A34" s="22"/>
       <c r="B34" s="11" t="s">
         <v>224</v>
@@ -28231,7 +28236,7 @@
         <v>1267</v>
       </c>
     </row>
-    <row r="35" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:62">
       <c r="A35" s="23"/>
       <c r="B35" s="13" t="s">
         <v>280</v>
@@ -28417,7 +28422,7 @@
         <v>1267</v>
       </c>
     </row>
-    <row r="36" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:62">
       <c r="A36" s="24" t="s">
         <v>1322</v>
       </c>
@@ -28605,7 +28610,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="37" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:62">
       <c r="A37" s="22"/>
       <c r="B37" s="11" t="s">
         <v>224</v>
@@ -28791,7 +28796,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="38" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:62">
       <c r="A38" s="23"/>
       <c r="B38" s="13" t="s">
         <v>280</v>
@@ -28977,7 +28982,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="39" spans="1:62" ht="45" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:62" ht="45">
       <c r="A39" s="24" t="s">
         <v>1325</v>
       </c>
@@ -29165,7 +29170,7 @@
         <v>1410</v>
       </c>
     </row>
-    <row r="40" spans="1:62" ht="30" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:62" ht="30">
       <c r="A40" s="22"/>
       <c r="B40" s="11" t="s">
         <v>224</v>
@@ -29351,7 +29356,7 @@
         <v>1400</v>
       </c>
     </row>
-    <row r="41" spans="1:62" ht="30" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:62" ht="30">
       <c r="A41" s="23"/>
       <c r="B41" s="13" t="s">
         <v>280</v>
@@ -29537,7 +29542,7 @@
         <v>1445</v>
       </c>
     </row>
-    <row r="42" spans="1:62" ht="45" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:62" ht="45">
       <c r="A42" s="24" t="s">
         <v>1455</v>
       </c>
@@ -29725,7 +29730,7 @@
         <v>1513</v>
       </c>
     </row>
-    <row r="43" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:62">
       <c r="A43" s="22"/>
       <c r="B43" s="11" t="s">
         <v>224</v>
@@ -29911,7 +29916,7 @@
         <v>1489</v>
       </c>
     </row>
-    <row r="44" spans="1:62" ht="30" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:62" ht="30">
       <c r="A44" s="23"/>
       <c r="B44" s="13" t="s">
         <v>280</v>
@@ -30097,7 +30102,7 @@
         <v>1526</v>
       </c>
     </row>
-    <row r="45" spans="1:62" ht="30" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:62" ht="30">
       <c r="A45" s="24" t="s">
         <v>1558</v>
       </c>
@@ -30285,7 +30290,7 @@
         <v>1569</v>
       </c>
     </row>
-    <row r="46" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:62">
       <c r="A46" s="22"/>
       <c r="B46" s="11" t="s">
         <v>224</v>
@@ -30471,7 +30476,7 @@
         <v>1591</v>
       </c>
     </row>
-    <row r="47" spans="1:62" ht="30" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:62" ht="30">
       <c r="A47" s="23"/>
       <c r="B47" s="13" t="s">
         <v>280</v>
@@ -30657,7 +30662,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="48" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:62">
       <c r="A48" s="24" t="s">
         <v>1616</v>
       </c>
@@ -30845,7 +30850,7 @@
         <v>1631</v>
       </c>
     </row>
-    <row r="49" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:62">
       <c r="A49" s="22"/>
       <c r="B49" s="11" t="s">
         <v>224</v>
@@ -31031,7 +31036,7 @@
         <v>1590</v>
       </c>
     </row>
-    <row r="50" spans="1:62" ht="30" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:62" ht="30">
       <c r="A50" s="23"/>
       <c r="B50" s="13" t="s">
         <v>280</v>
@@ -31217,7 +31222,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="51" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:62">
       <c r="A51" s="24" t="s">
         <v>1653</v>
       </c>
@@ -31405,7 +31410,7 @@
         <v>1267</v>
       </c>
     </row>
-    <row r="52" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:62">
       <c r="A52" s="22"/>
       <c r="B52" s="11" t="s">
         <v>224</v>
@@ -31591,7 +31596,7 @@
         <v>1267</v>
       </c>
     </row>
-    <row r="53" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:62">
       <c r="A53" s="23"/>
       <c r="B53" s="13" t="s">
         <v>280</v>
@@ -31777,7 +31782,7 @@
         <v>1267</v>
       </c>
     </row>
-    <row r="54" spans="1:62" ht="30" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:62" ht="30">
       <c r="A54" s="24" t="s">
         <v>1655</v>
       </c>
@@ -31965,7 +31970,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="55" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:62">
       <c r="A55" s="22"/>
       <c r="B55" s="11" t="s">
         <v>224</v>
@@ -32151,7 +32156,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="56" spans="1:62" ht="30" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:62" ht="30">
       <c r="A56" s="23"/>
       <c r="B56" s="13" t="s">
         <v>280</v>
@@ -32337,7 +32342,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="57" spans="1:62" ht="135" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:62" ht="135">
       <c r="A57" s="24" t="s">
         <v>1678</v>
       </c>
@@ -32525,7 +32530,7 @@
         <v>1801</v>
       </c>
     </row>
-    <row r="58" spans="1:62" ht="120" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:62" ht="120">
       <c r="A58" s="22"/>
       <c r="B58" s="11" t="s">
         <v>224</v>
@@ -32711,7 +32716,7 @@
         <v>1859</v>
       </c>
     </row>
-    <row r="59" spans="1:62" ht="195" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:62" ht="195">
       <c r="A59" s="23"/>
       <c r="B59" s="13" t="s">
         <v>280</v>
@@ -32899,6 +32904,15 @@
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="A6:A8"/>
+    <mergeCell ref="A3:A5"/>
+    <mergeCell ref="A42:A44"/>
+    <mergeCell ref="A18:A20"/>
+    <mergeCell ref="A27:A29"/>
+    <mergeCell ref="A9:A11"/>
+    <mergeCell ref="A36:A38"/>
+    <mergeCell ref="A30:A32"/>
+    <mergeCell ref="A39:A41"/>
     <mergeCell ref="A45:A47"/>
     <mergeCell ref="A21:A23"/>
     <mergeCell ref="A12:A14"/>
@@ -32909,32 +32923,27 @@
     <mergeCell ref="A48:A50"/>
     <mergeCell ref="A51:A53"/>
     <mergeCell ref="A54:A56"/>
-    <mergeCell ref="A6:A8"/>
-    <mergeCell ref="A3:A5"/>
-    <mergeCell ref="A42:A44"/>
-    <mergeCell ref="A18:A20"/>
-    <mergeCell ref="A27:A29"/>
-    <mergeCell ref="A9:A11"/>
-    <mergeCell ref="A36:A38"/>
-    <mergeCell ref="A30:A32"/>
-    <mergeCell ref="A39:A41"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:BJ97"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="28" customWidth="1"/>
-    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="1" max="1" width="12.5" customWidth="1"/>
+    <col min="2" max="2" width="9.6640625" customWidth="1"/>
     <col min="3" max="62" width="36" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:62" ht="25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:62" ht="25" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -33122,7 +33131,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="2" spans="1:62" ht="140" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:62" ht="140" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>62</v>
       </c>
@@ -33190,7 +33199,7 @@
       <c r="BI2" s="4"/>
       <c r="BJ2" s="4"/>
     </row>
-    <row r="3" spans="1:62" ht="45" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:62" ht="45">
       <c r="A3" s="21" t="s">
         <v>64</v>
       </c>
@@ -33378,7 +33387,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="4" spans="1:62" ht="75" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:62" ht="75">
       <c r="A4" s="22"/>
       <c r="B4" s="7" t="s">
         <v>121</v>
@@ -33564,7 +33573,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="5" spans="1:62" ht="45" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:62" ht="45">
       <c r="A5" s="22"/>
       <c r="B5" s="9" t="s">
         <v>174</v>
@@ -33750,7 +33759,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="6" spans="1:62" ht="45" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:62" ht="45">
       <c r="A6" s="22"/>
       <c r="B6" s="11" t="s">
         <v>224</v>
@@ -33936,7 +33945,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="7" spans="1:62" ht="30" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:62" ht="30">
       <c r="A7" s="23"/>
       <c r="B7" s="13" t="s">
         <v>280</v>
@@ -34122,7 +34131,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="8" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:62">
       <c r="A8" s="21" t="s">
         <v>324</v>
       </c>
@@ -34310,7 +34319,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="9" spans="1:62" ht="45" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:62" ht="45">
       <c r="A9" s="22"/>
       <c r="B9" s="7" t="s">
         <v>121</v>
@@ -34496,7 +34505,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="10" spans="1:62" ht="30" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:62" ht="30">
       <c r="A10" s="22"/>
       <c r="B10" s="9" t="s">
         <v>174</v>
@@ -34682,7 +34691,7 @@
         <v>461</v>
       </c>
     </row>
-    <row r="11" spans="1:62" ht="30" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:62" ht="30">
       <c r="A11" s="22"/>
       <c r="B11" s="11" t="s">
         <v>224</v>
@@ -34868,7 +34877,7 @@
         <v>502</v>
       </c>
     </row>
-    <row r="12" spans="1:62" ht="60" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:62" ht="60">
       <c r="A12" s="23"/>
       <c r="B12" s="13" t="s">
         <v>280</v>
@@ -35054,7 +35063,7 @@
         <v>559</v>
       </c>
     </row>
-    <row r="13" spans="1:62" ht="30" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:62" ht="30">
       <c r="A13" s="21" t="s">
         <v>560</v>
       </c>
@@ -35242,7 +35251,7 @@
         <v>570</v>
       </c>
     </row>
-    <row r="14" spans="1:62" ht="30" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:62" ht="30">
       <c r="A14" s="22"/>
       <c r="B14" s="7" t="s">
         <v>121</v>
@@ -35428,7 +35437,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="15" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:62">
       <c r="A15" s="22"/>
       <c r="B15" s="9" t="s">
         <v>174</v>
@@ -35614,7 +35623,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="16" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:62">
       <c r="A16" s="22"/>
       <c r="B16" s="11" t="s">
         <v>224</v>
@@ -35800,7 +35809,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="17" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:62">
       <c r="A17" s="23"/>
       <c r="B17" s="13" t="s">
         <v>280</v>
@@ -35986,7 +35995,7 @@
         <v>610</v>
       </c>
     </row>
-    <row r="18" spans="1:62" ht="45" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:62" ht="45">
       <c r="A18" s="21" t="s">
         <v>611</v>
       </c>
@@ -36174,7 +36183,7 @@
         <v>648</v>
       </c>
     </row>
-    <row r="19" spans="1:62" ht="75" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:62" ht="75">
       <c r="A19" s="22"/>
       <c r="B19" s="7" t="s">
         <v>121</v>
@@ -36360,7 +36369,7 @@
         <v>698</v>
       </c>
     </row>
-    <row r="20" spans="1:62" ht="75" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:62" ht="60">
       <c r="A20" s="22"/>
       <c r="B20" s="9" t="s">
         <v>174</v>
@@ -36546,7 +36555,7 @@
         <v>758</v>
       </c>
     </row>
-    <row r="21" spans="1:62" ht="60" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:62" ht="60">
       <c r="A21" s="22"/>
       <c r="B21" s="11" t="s">
         <v>224</v>
@@ -36732,7 +36741,7 @@
         <v>816</v>
       </c>
     </row>
-    <row r="22" spans="1:62" ht="120" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:62" ht="120">
       <c r="A22" s="23"/>
       <c r="B22" s="13" t="s">
         <v>280</v>
@@ -36918,7 +36927,7 @@
         <v>876</v>
       </c>
     </row>
-    <row r="23" spans="1:62" ht="30" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:62" ht="30">
       <c r="A23" s="21" t="s">
         <v>877</v>
       </c>
@@ -37106,7 +37115,7 @@
         <v>885</v>
       </c>
     </row>
-    <row r="24" spans="1:62" ht="30" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:62" ht="30">
       <c r="A24" s="22"/>
       <c r="B24" s="7" t="s">
         <v>121</v>
@@ -37292,7 +37301,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="25" spans="1:62" ht="30" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:62" ht="30">
       <c r="A25" s="22"/>
       <c r="B25" s="9" t="s">
         <v>174</v>
@@ -37478,7 +37487,7 @@
         <v>903</v>
       </c>
     </row>
-    <row r="26" spans="1:62" ht="30" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:62" ht="30">
       <c r="A26" s="22"/>
       <c r="B26" s="11" t="s">
         <v>224</v>
@@ -37664,7 +37673,7 @@
         <v>904</v>
       </c>
     </row>
-    <row r="27" spans="1:62" ht="30" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:62" ht="30">
       <c r="A27" s="23"/>
       <c r="B27" s="13" t="s">
         <v>280</v>
@@ -37850,7 +37859,7 @@
         <v>904</v>
       </c>
     </row>
-    <row r="28" spans="1:62" ht="45" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:62" ht="45">
       <c r="A28" s="21" t="s">
         <v>924</v>
       </c>
@@ -38038,7 +38047,7 @@
         <v>926</v>
       </c>
     </row>
-    <row r="29" spans="1:62" ht="45" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:62" ht="45">
       <c r="A29" s="22"/>
       <c r="B29" s="7" t="s">
         <v>121</v>
@@ -38224,7 +38233,7 @@
         <v>925</v>
       </c>
     </row>
-    <row r="30" spans="1:62" ht="60" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:62" ht="60">
       <c r="A30" s="22"/>
       <c r="B30" s="9" t="s">
         <v>174</v>
@@ -38410,7 +38419,7 @@
         <v>957</v>
       </c>
     </row>
-    <row r="31" spans="1:62" ht="45" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:62" ht="45">
       <c r="A31" s="22"/>
       <c r="B31" s="11" t="s">
         <v>224</v>
@@ -38596,7 +38605,7 @@
         <v>954</v>
       </c>
     </row>
-    <row r="32" spans="1:62" ht="60" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:62" ht="60">
       <c r="A32" s="23"/>
       <c r="B32" s="13" t="s">
         <v>280</v>
@@ -38782,7 +38791,7 @@
         <v>954</v>
       </c>
     </row>
-    <row r="33" spans="1:62" ht="30" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:62" ht="30">
       <c r="A33" s="21" t="s">
         <v>971</v>
       </c>
@@ -38970,7 +38979,7 @@
         <v>997</v>
       </c>
     </row>
-    <row r="34" spans="1:62" ht="45" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:62" ht="45">
       <c r="A34" s="22"/>
       <c r="B34" s="7" t="s">
         <v>121</v>
@@ -39156,7 +39165,7 @@
         <v>1027</v>
       </c>
     </row>
-    <row r="35" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:62">
       <c r="A35" s="22"/>
       <c r="B35" s="9" t="s">
         <v>174</v>
@@ -39342,7 +39351,7 @@
         <v>1030</v>
       </c>
     </row>
-    <row r="36" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:62">
       <c r="A36" s="22"/>
       <c r="B36" s="11" t="s">
         <v>224</v>
@@ -39528,7 +39537,7 @@
         <v>1030</v>
       </c>
     </row>
-    <row r="37" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:62">
       <c r="A37" s="23"/>
       <c r="B37" s="13" t="s">
         <v>280</v>
@@ -39714,7 +39723,7 @@
         <v>1030</v>
       </c>
     </row>
-    <row r="38" spans="1:62" ht="60" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:62" ht="60">
       <c r="A38" s="21" t="s">
         <v>1033</v>
       </c>
@@ -39902,7 +39911,7 @@
         <v>1050</v>
       </c>
     </row>
-    <row r="39" spans="1:62" ht="150" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:62" ht="150">
       <c r="A39" s="22"/>
       <c r="B39" s="7" t="s">
         <v>121</v>
@@ -40088,7 +40097,7 @@
         <v>1105</v>
       </c>
     </row>
-    <row r="40" spans="1:62" ht="60" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:62" ht="60">
       <c r="A40" s="22"/>
       <c r="B40" s="9" t="s">
         <v>174</v>
@@ -40274,7 +40283,7 @@
         <v>1153</v>
       </c>
     </row>
-    <row r="41" spans="1:62" ht="60" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:62" ht="60">
       <c r="A41" s="22"/>
       <c r="B41" s="11" t="s">
         <v>224</v>
@@ -40460,7 +40469,7 @@
         <v>1210</v>
       </c>
     </row>
-    <row r="42" spans="1:62" ht="75" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:62" ht="75">
       <c r="A42" s="23"/>
       <c r="B42" s="13" t="s">
         <v>280</v>
@@ -40646,7 +40655,7 @@
         <v>1262</v>
       </c>
     </row>
-    <row r="43" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:62">
       <c r="A43" s="21" t="s">
         <v>1263</v>
       </c>
@@ -40834,7 +40843,7 @@
         <v>1264</v>
       </c>
     </row>
-    <row r="44" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:62">
       <c r="A44" s="22"/>
       <c r="B44" s="7" t="s">
         <v>121</v>
@@ -41020,7 +41029,7 @@
         <v>1264</v>
       </c>
     </row>
-    <row r="45" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:62">
       <c r="A45" s="22"/>
       <c r="B45" s="9" t="s">
         <v>174</v>
@@ -41206,7 +41215,7 @@
         <v>1266</v>
       </c>
     </row>
-    <row r="46" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:62">
       <c r="A46" s="22"/>
       <c r="B46" s="11" t="s">
         <v>224</v>
@@ -41392,7 +41401,7 @@
         <v>1266</v>
       </c>
     </row>
-    <row r="47" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:62">
       <c r="A47" s="23"/>
       <c r="B47" s="13" t="s">
         <v>280</v>
@@ -41578,7 +41587,7 @@
         <v>1266</v>
       </c>
     </row>
-    <row r="48" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:62">
       <c r="A48" s="21" t="s">
         <v>1268</v>
       </c>
@@ -41766,7 +41775,7 @@
         <v>1278</v>
       </c>
     </row>
-    <row r="49" spans="1:62" ht="30" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:62" ht="30">
       <c r="A49" s="22"/>
       <c r="B49" s="7" t="s">
         <v>121</v>
@@ -41952,7 +41961,7 @@
         <v>1293</v>
       </c>
     </row>
-    <row r="50" spans="1:62" ht="30" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:62" ht="30">
       <c r="A50" s="22"/>
       <c r="B50" s="9" t="s">
         <v>174</v>
@@ -42138,7 +42147,7 @@
         <v>1301</v>
       </c>
     </row>
-    <row r="51" spans="1:62" ht="30" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:62" ht="30">
       <c r="A51" s="22"/>
       <c r="B51" s="11" t="s">
         <v>224</v>
@@ -42324,7 +42333,7 @@
         <v>1302</v>
       </c>
     </row>
-    <row r="52" spans="1:62" ht="45" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:62" ht="45">
       <c r="A52" s="23"/>
       <c r="B52" s="13" t="s">
         <v>280</v>
@@ -42510,7 +42519,7 @@
         <v>1301</v>
       </c>
     </row>
-    <row r="53" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:62">
       <c r="A53" s="21" t="s">
         <v>1321</v>
       </c>
@@ -42698,7 +42707,7 @@
         <v>1265</v>
       </c>
     </row>
-    <row r="54" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:62">
       <c r="A54" s="22"/>
       <c r="B54" s="7" t="s">
         <v>121</v>
@@ -42884,7 +42893,7 @@
         <v>1264</v>
       </c>
     </row>
-    <row r="55" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:62">
       <c r="A55" s="22"/>
       <c r="B55" s="9" t="s">
         <v>174</v>
@@ -43070,7 +43079,7 @@
         <v>1267</v>
       </c>
     </row>
-    <row r="56" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:62">
       <c r="A56" s="22"/>
       <c r="B56" s="11" t="s">
         <v>224</v>
@@ -43256,7 +43265,7 @@
         <v>1267</v>
       </c>
     </row>
-    <row r="57" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:62">
       <c r="A57" s="23"/>
       <c r="B57" s="13" t="s">
         <v>280</v>
@@ -43442,7 +43451,7 @@
         <v>1267</v>
       </c>
     </row>
-    <row r="58" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:62">
       <c r="A58" s="21" t="s">
         <v>1322</v>
       </c>
@@ -43630,7 +43639,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="59" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:62">
       <c r="A59" s="22"/>
       <c r="B59" s="7" t="s">
         <v>121</v>
@@ -43816,7 +43825,7 @@
         <v>1324</v>
       </c>
     </row>
-    <row r="60" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:62">
       <c r="A60" s="22"/>
       <c r="B60" s="9" t="s">
         <v>174</v>
@@ -44002,7 +44011,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="61" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:62">
       <c r="A61" s="22"/>
       <c r="B61" s="11" t="s">
         <v>224</v>
@@ -44188,7 +44197,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="62" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:62">
       <c r="A62" s="23"/>
       <c r="B62" s="13" t="s">
         <v>280</v>
@@ -44374,7 +44383,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="63" spans="1:62" ht="30" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:62" ht="30">
       <c r="A63" s="21" t="s">
         <v>1325</v>
       </c>
@@ -44562,7 +44571,7 @@
         <v>1326</v>
       </c>
     </row>
-    <row r="64" spans="1:62" ht="30" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:62" ht="30">
       <c r="A64" s="22"/>
       <c r="B64" s="7" t="s">
         <v>121</v>
@@ -44748,7 +44757,7 @@
         <v>1354</v>
       </c>
     </row>
-    <row r="65" spans="1:62" ht="45" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:62" ht="45">
       <c r="A65" s="22"/>
       <c r="B65" s="9" t="s">
         <v>174</v>
@@ -44934,7 +44943,7 @@
         <v>1410</v>
       </c>
     </row>
-    <row r="66" spans="1:62" ht="30" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:62" ht="30">
       <c r="A66" s="22"/>
       <c r="B66" s="11" t="s">
         <v>224</v>
@@ -45120,7 +45129,7 @@
         <v>1400</v>
       </c>
     </row>
-    <row r="67" spans="1:62" ht="30" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:62" ht="30">
       <c r="A67" s="23"/>
       <c r="B67" s="13" t="s">
         <v>280</v>
@@ -45306,7 +45315,7 @@
         <v>1445</v>
       </c>
     </row>
-    <row r="68" spans="1:62" ht="30" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:62" ht="30">
       <c r="A68" s="21" t="s">
         <v>1455</v>
       </c>
@@ -45494,7 +45503,7 @@
         <v>1338</v>
       </c>
     </row>
-    <row r="69" spans="1:62" ht="30" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:62" ht="30">
       <c r="A69" s="22"/>
       <c r="B69" s="7" t="s">
         <v>121</v>
@@ -45680,7 +45689,7 @@
         <v>1475</v>
       </c>
     </row>
-    <row r="70" spans="1:62" ht="45" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:62" ht="45">
       <c r="A70" s="22"/>
       <c r="B70" s="9" t="s">
         <v>174</v>
@@ -45866,7 +45875,7 @@
         <v>1513</v>
       </c>
     </row>
-    <row r="71" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:62">
       <c r="A71" s="22"/>
       <c r="B71" s="11" t="s">
         <v>224</v>
@@ -46052,7 +46061,7 @@
         <v>1489</v>
       </c>
     </row>
-    <row r="72" spans="1:62" ht="30" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:62" ht="30">
       <c r="A72" s="23"/>
       <c r="B72" s="13" t="s">
         <v>280</v>
@@ -46238,7 +46247,7 @@
         <v>1526</v>
       </c>
     </row>
-    <row r="73" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:62">
       <c r="A73" s="21" t="s">
         <v>1558</v>
       </c>
@@ -46426,7 +46435,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="74" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:62">
       <c r="A74" s="22"/>
       <c r="B74" s="7" t="s">
         <v>121</v>
@@ -46612,7 +46621,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="75" spans="1:62" ht="30" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:62" ht="30">
       <c r="A75" s="22"/>
       <c r="B75" s="9" t="s">
         <v>174</v>
@@ -46798,7 +46807,7 @@
         <v>1569</v>
       </c>
     </row>
-    <row r="76" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:62">
       <c r="A76" s="22"/>
       <c r="B76" s="11" t="s">
         <v>224</v>
@@ -46984,7 +46993,7 @@
         <v>1591</v>
       </c>
     </row>
-    <row r="77" spans="1:62" ht="30" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:62" ht="30">
       <c r="A77" s="23"/>
       <c r="B77" s="13" t="s">
         <v>280</v>
@@ -47170,7 +47179,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="78" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:62">
       <c r="A78" s="21" t="s">
         <v>1616</v>
       </c>
@@ -47358,7 +47367,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="79" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:62">
       <c r="A79" s="22"/>
       <c r="B79" s="7" t="s">
         <v>121</v>
@@ -47544,7 +47553,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="80" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:62">
       <c r="A80" s="22"/>
       <c r="B80" s="9" t="s">
         <v>174</v>
@@ -47730,7 +47739,7 @@
         <v>1631</v>
       </c>
     </row>
-    <row r="81" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:62">
       <c r="A81" s="22"/>
       <c r="B81" s="11" t="s">
         <v>224</v>
@@ -47916,7 +47925,7 @@
         <v>1590</v>
       </c>
     </row>
-    <row r="82" spans="1:62" ht="30" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:62" ht="30">
       <c r="A82" s="23"/>
       <c r="B82" s="13" t="s">
         <v>280</v>
@@ -48102,7 +48111,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="83" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:62">
       <c r="A83" s="21" t="s">
         <v>1653</v>
       </c>
@@ -48290,7 +48299,7 @@
         <v>1265</v>
       </c>
     </row>
-    <row r="84" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:62">
       <c r="A84" s="22"/>
       <c r="B84" s="7" t="s">
         <v>121</v>
@@ -48476,7 +48485,7 @@
         <v>1265</v>
       </c>
     </row>
-    <row r="85" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:62">
       <c r="A85" s="22"/>
       <c r="B85" s="9" t="s">
         <v>174</v>
@@ -48662,7 +48671,7 @@
         <v>1267</v>
       </c>
     </row>
-    <row r="86" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:62">
       <c r="A86" s="22"/>
       <c r="B86" s="11" t="s">
         <v>224</v>
@@ -48848,7 +48857,7 @@
         <v>1267</v>
       </c>
     </row>
-    <row r="87" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:62">
       <c r="A87" s="23"/>
       <c r="B87" s="13" t="s">
         <v>280</v>
@@ -49034,7 +49043,7 @@
         <v>1267</v>
       </c>
     </row>
-    <row r="88" spans="1:62" ht="30" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:62" ht="30">
       <c r="A88" s="21" t="s">
         <v>1655</v>
       </c>
@@ -49222,7 +49231,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="89" spans="1:62" ht="45" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:62" ht="45">
       <c r="A89" s="22"/>
       <c r="B89" s="7" t="s">
         <v>121</v>
@@ -49408,7 +49417,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="90" spans="1:62" ht="30" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:62" ht="30">
       <c r="A90" s="22"/>
       <c r="B90" s="9" t="s">
         <v>174</v>
@@ -49594,7 +49603,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="91" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:62">
       <c r="A91" s="22"/>
       <c r="B91" s="11" t="s">
         <v>224</v>
@@ -49780,7 +49789,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="92" spans="1:62" ht="30" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:62" ht="30">
       <c r="A92" s="23"/>
       <c r="B92" s="13" t="s">
         <v>280</v>
@@ -49966,7 +49975,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="93" spans="1:62" ht="75" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:62" ht="75">
       <c r="A93" s="21" t="s">
         <v>1678</v>
       </c>
@@ -50154,7 +50163,7 @@
         <v>1705</v>
       </c>
     </row>
-    <row r="94" spans="1:62" ht="105" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:62" ht="105">
       <c r="A94" s="22"/>
       <c r="B94" s="7" t="s">
         <v>121</v>
@@ -50340,7 +50349,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="95" spans="1:62" ht="135" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:62" ht="135">
       <c r="A95" s="22"/>
       <c r="B95" s="9" t="s">
         <v>174</v>
@@ -50526,7 +50535,7 @@
         <v>1801</v>
       </c>
     </row>
-    <row r="96" spans="1:62" ht="120" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:62" ht="120">
       <c r="A96" s="22"/>
       <c r="B96" s="11" t="s">
         <v>224</v>
@@ -50712,7 +50721,7 @@
         <v>1859</v>
       </c>
     </row>
-    <row r="97" spans="1:62" ht="195" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:62" ht="195">
       <c r="A97" s="23"/>
       <c r="B97" s="13" t="s">
         <v>280</v>
@@ -50900,6 +50909,9 @@
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="A8:A12"/>
+    <mergeCell ref="A33:A37"/>
+    <mergeCell ref="A23:A27"/>
     <mergeCell ref="A63:A67"/>
     <mergeCell ref="A28:A32"/>
     <mergeCell ref="A13:A17"/>
@@ -50916,11 +50928,10 @@
     <mergeCell ref="A38:A42"/>
     <mergeCell ref="A83:A87"/>
     <mergeCell ref="A18:A22"/>
-    <mergeCell ref="A8:A12"/>
-    <mergeCell ref="A33:A37"/>
-    <mergeCell ref="A23:A27"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.2" right="0" top="0.2" bottom="0.2" header="0" footer="0"/>
+  <pageSetup paperSize="9" scale="31" fitToWidth="6" fitToHeight="2" orientation="landscape" horizontalDpi="0" verticalDpi="0"/>
+  <headerFooter scaleWithDoc="0" alignWithMargins="0"/>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>